<commit_message>
chore(misc/security): redact hardcoded API keys, outreach enrich, freee invoice, contract master
</commit_message>
<xml_diff>
--- a/contract/契約マスター_v6.xlsx
+++ b/contract/契約マスター_v6.xlsx
@@ -2051,7 +2051,7 @@
       </c>
       <c r="C12" s="109" t="inlineStr">
         <is>
-          <t>5月末終了</t>
+          <t>稼働中</t>
         </is>
       </c>
       <c r="D12" s="110" t="inlineStr">
@@ -3702,7 +3702,7 @@
       </c>
       <c r="C36" s="101" t="inlineStr">
         <is>
-          <t>入場前</t>
+          <t>稼働中</t>
         </is>
       </c>
       <c r="D36" s="101" t="inlineStr">
@@ -5909,33 +5909,7 @@
         </is>
       </c>
     </row>
-    <row r="14" ht="21.75" customHeight="1" s="102">
-      <c r="B14" t="inlineStr">
-        <is>
-          <t>稼働中</t>
-        </is>
-      </c>
-      <c r="C14" t="inlineStr">
-        <is>
-          <t>鶴川</t>
-        </is>
-      </c>
-      <c r="D14" t="inlineStr">
-        <is>
-          <t>2026/5</t>
-        </is>
-      </c>
-      <c r="E14" t="inlineStr">
-        <is>
-          <t>長期</t>
-        </is>
-      </c>
-      <c r="F14" t="inlineStr">
-        <is>
-          <t>（確認中）</t>
-        </is>
-      </c>
-    </row>
+    <row r="14" ht="21.75" customHeight="1" s="102"/>
     <row r="15">
       <c r="A15" s="129" t="inlineStr">
         <is>

</xml_diff>